<commit_message>
Add accounting imports and workflow tools
</commit_message>
<xml_diff>
--- a/ventas_entrada.xlsx
+++ b/ventas_entrada.xlsx
@@ -1,53 +1,92 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Desarrollo\proyectos\automatizador-reportes\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1D17D1D-1598-40B9-8290-6C123A714DC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>producto</t>
-  </si>
-  <si>
-    <t>unidades</t>
-  </si>
-  <si>
-    <t>precio_unitario</t>
-  </si>
-  <si>
-    <t>Teclado</t>
-  </si>
-  <si>
-    <t>Mouse</t>
-  </si>
-  <si>
-    <t>Monitor</t>
-  </si>
-  <si>
-    <t>Auriculares</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+  <si>
+    <t>fecha</t>
+  </si>
+  <si>
+    <t>tipo_comprobante</t>
+  </si>
+  <si>
+    <t>punto_venta</t>
+  </si>
+  <si>
+    <t>numero</t>
+  </si>
+  <si>
+    <t>cuit</t>
+  </si>
+  <si>
+    <t>razon_social</t>
+  </si>
+  <si>
+    <t>operacion</t>
+  </si>
+  <si>
+    <t>neto_gravado</t>
+  </si>
+  <si>
+    <t>alicuota</t>
+  </si>
+  <si>
+    <t>iva</t>
+  </si>
+  <si>
+    <t>no_gravado_exento</t>
+  </si>
+  <si>
+    <t>percepciones</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>2026-09-03</t>
+  </si>
+  <si>
+    <t>2026-09-08</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>30712345671</t>
+  </si>
+  <si>
+    <t>30776543213</t>
+  </si>
+  <si>
+    <t>Proveedor Sintético Uno</t>
+  </si>
+  <si>
+    <t>Cliente Sintético Dos</t>
+  </si>
+  <si>
+    <t>ventas</t>
+  </si>
+  <si>
+    <t>compras</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,14 +123,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -379,14 +410,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9760CBC-DBDD-4C75-BBDE-CD3021DAACE6}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="3" max="3" width="13.5546875" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -396,49 +424,117 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2">
-        <v>5</v>
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
       </c>
       <c r="C2">
-        <v>12000</v>
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>101</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2">
+        <v>100000</v>
+      </c>
+      <c r="I2">
+        <v>21</v>
+      </c>
+      <c r="J2">
+        <v>21000</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>121000</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3">
-        <v>8</v>
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
       </c>
       <c r="C3">
-        <v>7500</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
         <v>2</v>
       </c>
-      <c r="C4">
-        <v>180000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5">
-        <v>25000</v>
+      <c r="D3">
+        <v>44</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3">
+        <v>50000</v>
+      </c>
+      <c r="I3">
+        <v>10.5</v>
+      </c>
+      <c r="J3">
+        <v>5250</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>55250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>